<commit_message>
SENDA: pendientes de prioridad baja, traducciones y estado de la lista
- PL4: alarmas en la zona horaria del teléfono (flutter_timezone); se reprograman si cambia.
- PL6: se quitan drift, sqlite3_flutter_libs, drift_dev y build_runner (sin uso).
- PL9: brillo al máximo mientras se muestra el QR (screen_brightness).
- SE7: con huella activa, tras 5 min en segundo plano se vuelve a pedir.
- A9: se documenta cuándo va C.marca y cuándo C.primary.
- A10: la voz y el audio avisan si fallan o falta la voz del idioma; pictograma sin red.
- PA7: la receta en PNG se sube como PNG.
- A6/T4: textos nuevos en textos_para_traducir.csv/.xlsx y prueba que exige inglés
  para todo tr('…') de lib/.
- docs/PENDIENTES_FRONTEND.md: estado de cada punto y propuestas para backend
  (registro y plan de control).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAwt2TWP4jaQGPM7PpqsGY
</commit_message>
<xml_diff>
--- a/docs/textos_para_traducir.xlsx
+++ b/docs/textos_para_traducir.xlsx
@@ -590,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F615"/>
+  <dimension ref="A1:F718"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -15733,6 +15733,2890 @@
       <c r="E615" s="7" t="inlineStr"/>
       <c r="F615" s="6" t="inlineStr"/>
     </row>
+    <row r="616">
+      <c r="A616" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B616" s="6" t="inlineStr">
+        <is>
+          <t>Confirma que eres tú para entrar a SENDA</t>
+        </is>
+      </c>
+      <c r="C616" s="6" t="inlineStr">
+        <is>
+          <t>Confirma que eres tú para entrar a SENDA</t>
+        </is>
+      </c>
+      <c r="D616" s="6" t="inlineStr">
+        <is>
+          <t>Confirm it is you to open SENDA</t>
+        </is>
+      </c>
+      <c r="E616" s="7" t="inlineStr"/>
+      <c r="F616" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B617" s="6" t="inlineStr">
+        <is>
+          <t>Este teléfono no tiene huella, rostro ni bloqueo de pantalla. Entra con tu contraseña.</t>
+        </is>
+      </c>
+      <c r="C617" s="6" t="inlineStr">
+        <is>
+          <t>Este teléfono no tiene huella, rostro ni bloqueo de pantalla. Entra con tu contraseña.</t>
+        </is>
+      </c>
+      <c r="D617" s="6" t="inlineStr">
+        <is>
+          <t>This phone has no fingerprint, face or screen lock. Log in with your password.</t>
+        </is>
+      </c>
+      <c r="E617" s="7" t="inlineStr"/>
+      <c r="F617" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B618" s="6" t="inlineStr">
+        <is>
+          <t>No hay huella ni rostro registrados en este teléfono. Regístralos en Ajustes o entra con tu contraseña.</t>
+        </is>
+      </c>
+      <c r="C618" s="6" t="inlineStr">
+        <is>
+          <t>No hay huella ni rostro registrados en este teléfono. Regístralos en Ajustes o entra con tu contraseña.</t>
+        </is>
+      </c>
+      <c r="D618" s="6" t="inlineStr">
+        <is>
+          <t>No fingerprint or face is registered on this phone. Add one in Settings or log in with your password.</t>
+        </is>
+      </c>
+      <c r="E618" s="7" t="inlineStr"/>
+      <c r="F618" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B619" s="6" t="inlineStr">
+        <is>
+          <t>Hubo demasiados intentos. Espera unos minutos o entra con tu contraseña.</t>
+        </is>
+      </c>
+      <c r="C619" s="6" t="inlineStr">
+        <is>
+          <t>Hubo demasiados intentos. Espera unos minutos o entra con tu contraseña.</t>
+        </is>
+      </c>
+      <c r="D619" s="6" t="inlineStr">
+        <is>
+          <t>Too many attempts. Wait a few minutes or log in with your password.</t>
+        </is>
+      </c>
+      <c r="E619" s="7" t="inlineStr"/>
+      <c r="F619" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B620" s="6" t="inlineStr">
+        <is>
+          <t>No se pudo confirmar tu identidad. Entra con tu contraseña.</t>
+        </is>
+      </c>
+      <c r="C620" s="6" t="inlineStr">
+        <is>
+          <t>No se pudo confirmar tu identidad. Entra con tu contraseña.</t>
+        </is>
+      </c>
+      <c r="D620" s="6" t="inlineStr">
+        <is>
+          <t>We could not confirm it is you. Log in with your password.</t>
+        </is>
+      </c>
+      <c r="E620" s="7" t="inlineStr"/>
+      <c r="F620" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B621" s="6" t="inlineStr">
+        <is>
+          <t>Entrar a SENDA</t>
+        </is>
+      </c>
+      <c r="C621" s="6" t="inlineStr">
+        <is>
+          <t>Entrar a SENDA</t>
+        </is>
+      </c>
+      <c r="D621" s="6" t="inlineStr">
+        <is>
+          <t>Open SENDA</t>
+        </is>
+      </c>
+      <c r="E621" s="7" t="inlineStr"/>
+      <c r="F621" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B622" s="6" t="inlineStr">
+        <is>
+          <t>Toca el sensor de huella o mira la cámara</t>
+        </is>
+      </c>
+      <c r="C622" s="6" t="inlineStr">
+        <is>
+          <t>Toca el sensor de huella o mira la cámara</t>
+        </is>
+      </c>
+      <c r="D622" s="6" t="inlineStr">
+        <is>
+          <t>Touch the fingerprint sensor or look at the camera</t>
+        </is>
+      </c>
+      <c r="E622" s="7" t="inlineStr"/>
+      <c r="F622" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B623" s="6" t="inlineStr">
+        <is>
+          <t>No se reconoció. Intenta de nuevo.</t>
+        </is>
+      </c>
+      <c r="C623" s="6" t="inlineStr">
+        <is>
+          <t>No se reconoció. Intenta de nuevo.</t>
+        </is>
+      </c>
+      <c r="D623" s="6" t="inlineStr">
+        <is>
+          <t>Not recognized. Try again.</t>
+        </is>
+      </c>
+      <c r="E623" s="7" t="inlineStr"/>
+      <c r="F623" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B624" s="6" t="inlineStr">
+        <is>
+          <t>Se necesita tu huella o rostro</t>
+        </is>
+      </c>
+      <c r="C624" s="6" t="inlineStr">
+        <is>
+          <t>Se necesita tu huella o rostro</t>
+        </is>
+      </c>
+      <c r="D624" s="6" t="inlineStr">
+        <is>
+          <t>Your fingerprint or face is needed</t>
+        </is>
+      </c>
+      <c r="E624" s="7" t="inlineStr"/>
+      <c r="F624" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B625" s="6" t="inlineStr">
+        <is>
+          <t>Se necesita el bloqueo de tu teléfono</t>
+        </is>
+      </c>
+      <c r="C625" s="6" t="inlineStr">
+        <is>
+          <t>Se necesita el bloqueo de tu teléfono</t>
+        </is>
+      </c>
+      <c r="D625" s="6" t="inlineStr">
+        <is>
+          <t>Your phone lock is needed</t>
+        </is>
+      </c>
+      <c r="E625" s="7" t="inlineStr"/>
+      <c r="F625" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B626" s="6" t="inlineStr">
+        <is>
+          <t>Configura un bloqueo de pantalla en los Ajustes del teléfono.</t>
+        </is>
+      </c>
+      <c r="C626" s="6" t="inlineStr">
+        <is>
+          <t>Configura un bloqueo de pantalla en los Ajustes del teléfono.</t>
+        </is>
+      </c>
+      <c r="D626" s="6" t="inlineStr">
+        <is>
+          <t>Set up a screen lock in your phone Settings.</t>
+        </is>
+      </c>
+      <c r="E626" s="7" t="inlineStr"/>
+      <c r="F626" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B627" s="6" t="inlineStr">
+        <is>
+          <t>Ir a Ajustes</t>
+        </is>
+      </c>
+      <c r="C627" s="6" t="inlineStr">
+        <is>
+          <t>Ir a Ajustes</t>
+        </is>
+      </c>
+      <c r="D627" s="6" t="inlineStr">
+        <is>
+          <t>Go to Settings</t>
+        </is>
+      </c>
+      <c r="E627" s="7" t="inlineStr"/>
+      <c r="F627" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B628" s="6" t="inlineStr">
+        <is>
+          <t>No hay huella ni rostro registrados. Regístralos en Ajustes &gt; Seguridad.</t>
+        </is>
+      </c>
+      <c r="C628" s="6" t="inlineStr">
+        <is>
+          <t>No hay huella ni rostro registrados. Regístralos en Ajustes &gt; Seguridad.</t>
+        </is>
+      </c>
+      <c r="D628" s="6" t="inlineStr">
+        <is>
+          <t>No fingerprint or face is registered. Add one in Settings &gt; Security.</t>
+        </is>
+      </c>
+      <c r="E628" s="7" t="inlineStr"/>
+      <c r="F628" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B629" s="6" t="inlineStr">
+        <is>
+          <t>Face ID o Touch ID está bloqueado. Bloquea y desbloquea el teléfono para activarlo.</t>
+        </is>
+      </c>
+      <c r="C629" s="6" t="inlineStr">
+        <is>
+          <t>Face ID o Touch ID está bloqueado. Bloquea y desbloquea el teléfono para activarlo.</t>
+        </is>
+      </c>
+      <c r="D629" s="6" t="inlineStr">
+        <is>
+          <t>Face ID or Touch ID is locked. Lock and unlock your phone to turn it back on.</t>
+        </is>
+      </c>
+      <c r="E629" s="7" t="inlineStr"/>
+      <c r="F629" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B630" s="6" t="inlineStr">
+        <is>
+          <t>No hay Face ID ni Touch ID configurado. Actívalo en Ajustes.</t>
+        </is>
+      </c>
+      <c r="C630" s="6" t="inlineStr">
+        <is>
+          <t>No hay Face ID ni Touch ID configurado. Actívalo en Ajustes.</t>
+        </is>
+      </c>
+      <c r="D630" s="6" t="inlineStr">
+        <is>
+          <t>Face ID or Touch ID is not set up. Turn it on in Settings.</t>
+        </is>
+      </c>
+      <c r="E630" s="7" t="inlineStr"/>
+      <c r="F630" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B631" s="6" t="inlineStr">
+        <is>
+          <t>Usar el código del teléfono</t>
+        </is>
+      </c>
+      <c r="C631" s="6" t="inlineStr">
+        <is>
+          <t>Usar el código del teléfono</t>
+        </is>
+      </c>
+      <c r="D631" s="6" t="inlineStr">
+        <is>
+          <t>Use phone passcode</t>
+        </is>
+      </c>
+      <c r="E631" s="7" t="inlineStr"/>
+      <c r="F631" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B632" s="6" t="inlineStr">
+        <is>
+          <t>Alertas de salud</t>
+        </is>
+      </c>
+      <c r="C632" s="6" t="inlineStr">
+        <is>
+          <t>Alertas de salud</t>
+        </is>
+      </c>
+      <c r="D632" s="6" t="inlineStr">
+        <is>
+          <t>Health alerts</t>
+        </is>
+      </c>
+      <c r="E632" s="7" t="inlineStr"/>
+      <c r="F632" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B633" s="6" t="inlineStr">
+        <is>
+          <t>Avisos del equipo de salud y de tus familiares.</t>
+        </is>
+      </c>
+      <c r="C633" s="6" t="inlineStr">
+        <is>
+          <t>Avisos del equipo de salud y de tus familiares.</t>
+        </is>
+      </c>
+      <c r="D633" s="6" t="inlineStr">
+        <is>
+          <t>Messages from your health team and your family.</t>
+        </is>
+      </c>
+      <c r="E633" s="7" t="inlineStr"/>
+      <c r="F633" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B634" s="6" t="inlineStr">
+        <is>
+          <t>Avisos y alarmas</t>
+        </is>
+      </c>
+      <c r="C634" s="6" t="inlineStr">
+        <is>
+          <t>Avisos y alarmas</t>
+        </is>
+      </c>
+      <c r="D634" s="6" t="inlineStr">
+        <is>
+          <t>Notifications and alarms</t>
+        </is>
+      </c>
+      <c r="E634" s="7" t="inlineStr"/>
+      <c r="F634" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B635" s="6" t="inlineStr">
+        <is>
+          <t>Permitidas.</t>
+        </is>
+      </c>
+      <c r="C635" s="6" t="inlineStr">
+        <is>
+          <t>Permitidas.</t>
+        </is>
+      </c>
+      <c r="D635" s="6" t="inlineStr">
+        <is>
+          <t>Allowed.</t>
+        </is>
+      </c>
+      <c r="E635" s="7" t="inlineStr"/>
+      <c r="F635" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B636" s="6" t="inlineStr">
+        <is>
+          <t>Desactivadas: no sonarán las alarmas de tus medicinas ni llegarán avisos.</t>
+        </is>
+      </c>
+      <c r="C636" s="6" t="inlineStr">
+        <is>
+          <t>Desactivadas: no sonarán las alarmas de tus medicinas ni llegarán avisos.</t>
+        </is>
+      </c>
+      <c r="D636" s="6" t="inlineStr">
+        <is>
+          <t>Turned off: your medicine alarms will not ring and you will not get messages.</t>
+        </is>
+      </c>
+      <c r="E636" s="7" t="inlineStr"/>
+      <c r="F636" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B637" s="6" t="inlineStr">
+        <is>
+          <t>Desactivadas: no llegarán los avisos de alertas.</t>
+        </is>
+      </c>
+      <c r="C637" s="6" t="inlineStr">
+        <is>
+          <t>Desactivadas: no llegarán los avisos de alertas.</t>
+        </is>
+      </c>
+      <c r="D637" s="6" t="inlineStr">
+        <is>
+          <t>Turned off: you will not get alert messages.</t>
+        </is>
+      </c>
+      <c r="E637" s="7" t="inlineStr"/>
+      <c r="F637" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B638" s="6" t="inlineStr">
+        <is>
+          <t>Permitir</t>
+        </is>
+      </c>
+      <c r="C638" s="6" t="inlineStr">
+        <is>
+          <t>Permitir</t>
+        </is>
+      </c>
+      <c r="D638" s="6" t="inlineStr">
+        <is>
+          <t>Allow</t>
+        </is>
+      </c>
+      <c r="E638" s="7" t="inlineStr"/>
+      <c r="F638" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B639" s="6" t="inlineStr">
+        <is>
+          <t>Alarmas a la hora exacta</t>
+        </is>
+      </c>
+      <c r="C639" s="6" t="inlineStr">
+        <is>
+          <t>Alarmas a la hora exacta</t>
+        </is>
+      </c>
+      <c r="D639" s="6" t="inlineStr">
+        <is>
+          <t>Alarms at the exact time</t>
+        </is>
+      </c>
+      <c r="E639" s="7" t="inlineStr"/>
+      <c r="F639" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B640" s="6" t="inlineStr">
+        <is>
+          <t>Activadas.</t>
+        </is>
+      </c>
+      <c r="C640" s="6" t="inlineStr">
+        <is>
+          <t>Activadas.</t>
+        </is>
+      </c>
+      <c r="D640" s="6" t="inlineStr">
+        <is>
+          <t>Turned on.</t>
+        </is>
+      </c>
+      <c r="E640" s="7" t="inlineStr"/>
+      <c r="F640" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B641" s="6" t="inlineStr">
+        <is>
+          <t>Las alarmas pueden sonar unos minutos tarde.</t>
+        </is>
+      </c>
+      <c r="C641" s="6" t="inlineStr">
+        <is>
+          <t>Las alarmas pueden sonar unos minutos tarde.</t>
+        </is>
+      </c>
+      <c r="D641" s="6" t="inlineStr">
+        <is>
+          <t>Alarms may ring a few minutes late.</t>
+        </is>
+      </c>
+      <c r="E641" s="7" t="inlineStr"/>
+      <c r="F641" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B642" s="6" t="inlineStr">
+        <is>
+          <t>Activar</t>
+        </is>
+      </c>
+      <c r="C642" s="6" t="inlineStr">
+        <is>
+          <t>Activar</t>
+        </is>
+      </c>
+      <c r="D642" s="6" t="inlineStr">
+        <is>
+          <t>Turn on</t>
+        </is>
+      </c>
+      <c r="E642" s="7" t="inlineStr"/>
+      <c r="F642" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B643" s="6" t="inlineStr">
+        <is>
+          <t>Alarma en pantalla completa</t>
+        </is>
+      </c>
+      <c r="C643" s="6" t="inlineStr">
+        <is>
+          <t>Alarma en pantalla completa</t>
+        </is>
+      </c>
+      <c r="D643" s="6" t="inlineStr">
+        <is>
+          <t>Full-screen alarm</t>
+        </is>
+      </c>
+      <c r="E643" s="7" t="inlineStr"/>
+      <c r="F643" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B644" s="6" t="inlineStr">
+        <is>
+          <t>La alarma aparece aunque el teléfono esté bloqueado.</t>
+        </is>
+      </c>
+      <c r="C644" s="6" t="inlineStr">
+        <is>
+          <t>La alarma aparece aunque el teléfono esté bloqueado.</t>
+        </is>
+      </c>
+      <c r="D644" s="6" t="inlineStr">
+        <is>
+          <t>The alarm shows up even when the phone is locked.</t>
+        </is>
+      </c>
+      <c r="E644" s="7" t="inlineStr"/>
+      <c r="F644" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B645" s="6" t="inlineStr">
+        <is>
+          <t>La alarma llegará como notificación, sin cubrir la pantalla.</t>
+        </is>
+      </c>
+      <c r="C645" s="6" t="inlineStr">
+        <is>
+          <t>La alarma llegará como notificación, sin cubrir la pantalla.</t>
+        </is>
+      </c>
+      <c r="D645" s="6" t="inlineStr">
+        <is>
+          <t>The alarm will arrive as a notification, without covering the screen.</t>
+        </is>
+      </c>
+      <c r="E645" s="7" t="inlineStr"/>
+      <c r="F645" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B646" s="6" t="inlineStr">
+        <is>
+          <t>Ahorro de batería</t>
+        </is>
+      </c>
+      <c r="C646" s="6" t="inlineStr">
+        <is>
+          <t>Ahorro de batería</t>
+        </is>
+      </c>
+      <c r="D646" s="6" t="inlineStr">
+        <is>
+          <t>Battery saver</t>
+        </is>
+      </c>
+      <c r="E646" s="7" t="inlineStr"/>
+      <c r="F646" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B647" s="6" t="inlineStr">
+        <is>
+          <t>Sin restricciones para SENDA.</t>
+        </is>
+      </c>
+      <c r="C647" s="6" t="inlineStr">
+        <is>
+          <t>Sin restricciones para SENDA.</t>
+        </is>
+      </c>
+      <c r="D647" s="6" t="inlineStr">
+        <is>
+          <t>No restrictions for SENDA.</t>
+        </is>
+      </c>
+      <c r="E647" s="7" t="inlineStr"/>
+      <c r="F647" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B648" s="6" t="inlineStr">
+        <is>
+          <t>El teléfono puede retrasar o silenciar las alarmas y avisos. Elige "Sin restricciones" para SENDA.</t>
+        </is>
+      </c>
+      <c r="C648" s="6" t="inlineStr">
+        <is>
+          <t>El teléfono puede retrasar o silenciar las alarmas y avisos. Elige "Sin restricciones" para SENDA.</t>
+        </is>
+      </c>
+      <c r="D648" s="6" t="inlineStr">
+        <is>
+          <t>The phone may delay or silence alarms and messages. Choose "Unrestricted" for SENDA.</t>
+        </is>
+      </c>
+      <c r="E648" s="7" t="inlineStr"/>
+      <c r="F648" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B649" s="6" t="inlineStr">
+        <is>
+          <t>En este teléfono activa también "Inicio automático" para SENDA.</t>
+        </is>
+      </c>
+      <c r="C649" s="6" t="inlineStr">
+        <is>
+          <t>En este teléfono activa también "Inicio automático" para SENDA.</t>
+        </is>
+      </c>
+      <c r="D649" s="6" t="inlineStr">
+        <is>
+          <t>On this phone also turn on "Autostart" for SENDA.</t>
+        </is>
+      </c>
+      <c r="E649" s="7" t="inlineStr"/>
+      <c r="F649" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B650" s="6" t="inlineStr">
+        <is>
+          <t>Abrir ajustes</t>
+        </is>
+      </c>
+      <c r="C650" s="6" t="inlineStr">
+        <is>
+          <t>Abrir ajustes</t>
+        </is>
+      </c>
+      <c r="D650" s="6" t="inlineStr">
+        <is>
+          <t>Open settings</t>
+        </is>
+      </c>
+      <c r="E650" s="7" t="inlineStr"/>
+      <c r="F650" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B651" s="6" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="C651" s="6" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="D651" s="6" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="E651" s="7" t="inlineStr"/>
+      <c r="F651" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B652" s="6" t="inlineStr">
+        <is>
+          <t>No se pudieron enviar</t>
+        </is>
+      </c>
+      <c r="C652" s="6" t="inlineStr">
+        <is>
+          <t>No se pudieron enviar</t>
+        </is>
+      </c>
+      <c r="D652" s="6" t="inlineStr">
+        <is>
+          <t>Could not be sent</t>
+        </is>
+      </c>
+      <c r="E652" s="7" t="inlineStr"/>
+      <c r="F652" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B653" s="6" t="inlineStr">
+        <is>
+          <t>Descartar</t>
+        </is>
+      </c>
+      <c r="C653" s="6" t="inlineStr">
+        <is>
+          <t>Descartar</t>
+        </is>
+      </c>
+      <c r="D653" s="6" t="inlineStr">
+        <is>
+          <t>Discard</t>
+        </is>
+      </c>
+      <c r="E653" s="7" t="inlineStr"/>
+      <c r="F653" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B654" s="6" t="inlineStr">
+        <is>
+          <t>Algunos datos no se pudieron enviar</t>
+        </is>
+      </c>
+      <c r="C654" s="6" t="inlineStr">
+        <is>
+          <t>Algunos datos no se pudieron enviar</t>
+        </is>
+      </c>
+      <c r="D654" s="6" t="inlineStr">
+        <is>
+          <t>Some data could not be sent</t>
+        </is>
+      </c>
+      <c r="E654" s="7" t="inlineStr"/>
+      <c r="F654" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B655" s="6" t="inlineStr">
+        <is>
+          <t>Por ahora las cuentas las crea tu equipo de salud. Pídeles tu usuario y contraseña.</t>
+        </is>
+      </c>
+      <c r="C655" s="6" t="inlineStr">
+        <is>
+          <t>Por ahora las cuentas las crea tu equipo de salud. Pídeles tu usuario y contraseña.</t>
+        </is>
+      </c>
+      <c r="D655" s="6" t="inlineStr">
+        <is>
+          <t>For now, accounts are created by your health team. Ask them for your username and password.</t>
+        </is>
+      </c>
+      <c r="E655" s="7" t="inlineStr"/>
+      <c r="F655" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B656" s="6" t="inlineStr">
+        <is>
+          <t>Ya existe una cuenta con ese correo. Inicia sesión.</t>
+        </is>
+      </c>
+      <c r="C656" s="6" t="inlineStr">
+        <is>
+          <t>Ya existe una cuenta con ese correo. Inicia sesión.</t>
+        </is>
+      </c>
+      <c r="D656" s="6" t="inlineStr">
+        <is>
+          <t>An account with that email already exists. Log in.</t>
+        </is>
+      </c>
+      <c r="E656" s="7" t="inlineStr"/>
+      <c r="F656" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B657" s="6" t="inlineStr">
+        <is>
+          <t>SENDA no tiene permiso de usar la cámara</t>
+        </is>
+      </c>
+      <c r="C657" s="6" t="inlineStr">
+        <is>
+          <t>SENDA no tiene permiso de usar la cámara</t>
+        </is>
+      </c>
+      <c r="D657" s="6" t="inlineStr">
+        <is>
+          <t>SENDA does not have permission to use the camera</t>
+        </is>
+      </c>
+      <c r="E657" s="7" t="inlineStr"/>
+      <c r="F657" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B658" s="6" t="inlineStr">
+        <is>
+          <t>SENDA no tiene permiso de ver tus fotos</t>
+        </is>
+      </c>
+      <c r="C658" s="6" t="inlineStr">
+        <is>
+          <t>SENDA no tiene permiso de ver tus fotos</t>
+        </is>
+      </c>
+      <c r="D658" s="6" t="inlineStr">
+        <is>
+          <t>SENDA does not have permission to see your photos</t>
+        </is>
+      </c>
+      <c r="E658" s="7" t="inlineStr"/>
+      <c r="F658" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B659" s="6" t="inlineStr">
+        <is>
+          <t>Para tomar la foto, permite la cámara en los Ajustes del teléfono y vuelve a intentarlo.</t>
+        </is>
+      </c>
+      <c r="C659" s="6" t="inlineStr">
+        <is>
+          <t>Para tomar la foto, permite la cámara en los Ajustes del teléfono y vuelve a intentarlo.</t>
+        </is>
+      </c>
+      <c r="D659" s="6" t="inlineStr">
+        <is>
+          <t>To take the photo, allow the camera in your phone Settings and try again.</t>
+        </is>
+      </c>
+      <c r="E659" s="7" t="inlineStr"/>
+      <c r="F659" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B660" s="6" t="inlineStr">
+        <is>
+          <t>Para elegir una foto, permite el acceso a fotos en los Ajustes del teléfono y vuelve a intentarlo.</t>
+        </is>
+      </c>
+      <c r="C660" s="6" t="inlineStr">
+        <is>
+          <t>Para elegir una foto, permite el acceso a fotos en los Ajustes del teléfono y vuelve a intentarlo.</t>
+        </is>
+      </c>
+      <c r="D660" s="6" t="inlineStr">
+        <is>
+          <t>To choose a photo, allow access to photos in your phone Settings and try again.</t>
+        </is>
+      </c>
+      <c r="E660" s="7" t="inlineStr"/>
+      <c r="F660" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B661" s="6" t="inlineStr">
+        <is>
+          <t>Ahora no</t>
+        </is>
+      </c>
+      <c r="C661" s="6" t="inlineStr">
+        <is>
+          <t>Ahora no</t>
+        </is>
+      </c>
+      <c r="D661" s="6" t="inlineStr">
+        <is>
+          <t>Not now</t>
+        </is>
+      </c>
+      <c r="E661" s="7" t="inlineStr"/>
+      <c r="F661" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B662" s="6" t="inlineStr">
+        <is>
+          <t>No se pudo abrir la cámara.</t>
+        </is>
+      </c>
+      <c r="C662" s="6" t="inlineStr">
+        <is>
+          <t>No se pudo abrir la cámara.</t>
+        </is>
+      </c>
+      <c r="D662" s="6" t="inlineStr">
+        <is>
+          <t>Could not open the camera.</t>
+        </is>
+      </c>
+      <c r="E662" s="7" t="inlineStr"/>
+      <c r="F662" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B663" s="6" t="inlineStr">
+        <is>
+          <t>No se pudo abrir la galería.</t>
+        </is>
+      </c>
+      <c r="C663" s="6" t="inlineStr">
+        <is>
+          <t>No se pudo abrir la galería.</t>
+        </is>
+      </c>
+      <c r="D663" s="6" t="inlineStr">
+        <is>
+          <t>Could not open the gallery.</t>
+        </is>
+      </c>
+      <c r="E663" s="7" t="inlineStr"/>
+      <c r="F663" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B664" s="6" t="inlineStr">
+        <is>
+          <t>SENDA no tiene permiso de usar la cámara. Permítelo en Ajustes o usa "Escribir código".</t>
+        </is>
+      </c>
+      <c r="C664" s="6" t="inlineStr">
+        <is>
+          <t>SENDA no tiene permiso de usar la cámara. Permítelo en Ajustes o usa "Escribir código".</t>
+        </is>
+      </c>
+      <c r="D664" s="6" t="inlineStr">
+        <is>
+          <t>SENDA does not have permission to use the camera. Allow it in Settings or use "Type code".</t>
+        </is>
+      </c>
+      <c r="E664" s="7" t="inlineStr"/>
+      <c r="F664" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B665" s="6" t="inlineStr">
+        <is>
+          <t>No se pudo abrir el teléfono. Marca al {n}.</t>
+        </is>
+      </c>
+      <c r="C665" s="6" t="inlineStr">
+        <is>
+          <t>No se pudo abrir el teléfono. Marca al {n}.</t>
+        </is>
+      </c>
+      <c r="D665" s="6" t="inlineStr">
+        <is>
+          <t>Could not open the phone app. Dial {n}.</t>
+        </is>
+      </c>
+      <c r="E665" s="7" t="inlineStr"/>
+      <c r="F665" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes). Conservar {…} tal cual: se reemplaza por un dato</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B666" s="6" t="inlineStr">
+        <is>
+          <t>Pedir ayuda</t>
+        </is>
+      </c>
+      <c r="C666" s="6" t="inlineStr">
+        <is>
+          <t>Pedir ayuda</t>
+        </is>
+      </c>
+      <c r="D666" s="6" t="inlineStr">
+        <is>
+          <t>Ask for help</t>
+        </is>
+      </c>
+      <c r="E666" s="7" t="inlineStr"/>
+      <c r="F666" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B667" s="6" t="inlineStr">
+        <is>
+          <t>No tenemos el teléfono de tu cuidador. Pide a tu equipo de salud que lo registre.</t>
+        </is>
+      </c>
+      <c r="C667" s="6" t="inlineStr">
+        <is>
+          <t>No tenemos el teléfono de tu cuidador. Pide a tu equipo de salud que lo registre.</t>
+        </is>
+      </c>
+      <c r="D667" s="6" t="inlineStr">
+        <is>
+          <t>We do not have your caregiver's phone number. Ask your health team to add it.</t>
+        </is>
+      </c>
+      <c r="E667" s="7" t="inlineStr"/>
+      <c r="F667" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B668" s="6" t="inlineStr">
+        <is>
+          <t>No tenemos el teléfono de {nombre}. Pide a tu equipo de salud que lo registre.</t>
+        </is>
+      </c>
+      <c r="C668" s="6" t="inlineStr">
+        <is>
+          <t>No tenemos el teléfono de {nombre}. Pide a tu equipo de salud que lo registre.</t>
+        </is>
+      </c>
+      <c r="D668" s="6" t="inlineStr">
+        <is>
+          <t>We do not have {nombre}'s phone number. Ask your health team to add it.</t>
+        </is>
+      </c>
+      <c r="E668" s="7" t="inlineStr"/>
+      <c r="F668" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes). Conservar {…} tal cual: se reemplaza por un dato</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B669" s="6" t="inlineStr">
+        <is>
+          <t>Vamos a llamar a {nombre} al {tel}.</t>
+        </is>
+      </c>
+      <c r="C669" s="6" t="inlineStr">
+        <is>
+          <t>Vamos a llamar a {nombre} al {tel}.</t>
+        </is>
+      </c>
+      <c r="D669" s="6" t="inlineStr">
+        <is>
+          <t>We will call {nombre} at {tel}.</t>
+        </is>
+      </c>
+      <c r="E669" s="7" t="inlineStr"/>
+      <c r="F669" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes). Conservar {…} tal cual: se reemplaza por un dato</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B670" s="6" t="inlineStr">
+        <is>
+          <t>tu cuidador</t>
+        </is>
+      </c>
+      <c r="C670" s="6" t="inlineStr">
+        <is>
+          <t>tu cuidador</t>
+        </is>
+      </c>
+      <c r="D670" s="6" t="inlineStr">
+        <is>
+          <t>your caregiver</t>
+        </is>
+      </c>
+      <c r="E670" s="7" t="inlineStr"/>
+      <c r="F670" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B671" s="6" t="inlineStr">
+        <is>
+          <t>Si te sientes muy mal, llama al 911.</t>
+        </is>
+      </c>
+      <c r="C671" s="6" t="inlineStr">
+        <is>
+          <t>Si te sientes muy mal, llama al 911.</t>
+        </is>
+      </c>
+      <c r="D671" s="6" t="inlineStr">
+        <is>
+          <t>If you feel very sick, call 911.</t>
+        </is>
+      </c>
+      <c r="E671" s="7" t="inlineStr"/>
+      <c r="F671" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B672" s="6" t="inlineStr">
+        <is>
+          <t>Llamar al 911</t>
+        </is>
+      </c>
+      <c r="C672" s="6" t="inlineStr">
+        <is>
+          <t>Llamar al 911</t>
+        </is>
+      </c>
+      <c r="D672" s="6" t="inlineStr">
+        <is>
+          <t>Call 911</t>
+        </is>
+      </c>
+      <c r="E672" s="7" t="inlineStr"/>
+      <c r="F672" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B673" s="6" t="inlineStr">
+        <is>
+          <t>Llamar a mi cuidador</t>
+        </is>
+      </c>
+      <c r="C673" s="6" t="inlineStr">
+        <is>
+          <t>Llamar a mi cuidador</t>
+        </is>
+      </c>
+      <c r="D673" s="6" t="inlineStr">
+        <is>
+          <t>Call my caregiver</t>
+        </is>
+      </c>
+      <c r="E673" s="7" t="inlineStr"/>
+      <c r="F673" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B674" s="6" t="inlineStr">
+        <is>
+          <t>Llamar a {nombre}</t>
+        </is>
+      </c>
+      <c r="C674" s="6" t="inlineStr">
+        <is>
+          <t>Llamar a {nombre}</t>
+        </is>
+      </c>
+      <c r="D674" s="6" t="inlineStr">
+        <is>
+          <t>Call {nombre}</t>
+        </is>
+      </c>
+      <c r="E674" s="7" t="inlineStr"/>
+      <c r="F674" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes). Conservar {…} tal cual: se reemplaza por un dato</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B675" s="6" t="inlineStr">
+        <is>
+          <t>Una vez al día</t>
+        </is>
+      </c>
+      <c r="C675" s="6" t="inlineStr">
+        <is>
+          <t>Una vez al día</t>
+        </is>
+      </c>
+      <c r="D675" s="6" t="inlineStr">
+        <is>
+          <t>Once a day</t>
+        </is>
+      </c>
+      <c r="E675" s="7" t="inlineStr"/>
+      <c r="F675" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B676" s="6" t="inlineStr">
+        <is>
+          <t>Dos veces al día</t>
+        </is>
+      </c>
+      <c r="C676" s="6" t="inlineStr">
+        <is>
+          <t>Dos veces al día</t>
+        </is>
+      </c>
+      <c r="D676" s="6" t="inlineStr">
+        <is>
+          <t>Twice a day</t>
+        </is>
+      </c>
+      <c r="E676" s="7" t="inlineStr"/>
+      <c r="F676" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B677" s="6" t="inlineStr">
+        <is>
+          <t>Una vez a la semana</t>
+        </is>
+      </c>
+      <c r="C677" s="6" t="inlineStr">
+        <is>
+          <t>Una vez a la semana</t>
+        </is>
+      </c>
+      <c r="D677" s="6" t="inlineStr">
+        <is>
+          <t>Once a week</t>
+        </is>
+      </c>
+      <c r="E677" s="7" t="inlineStr"/>
+      <c r="F677" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B678" s="6" t="inlineStr">
+        <is>
+          <t>{v}: escribe el mínimo y el máximo{e}.</t>
+        </is>
+      </c>
+      <c r="C678" s="6" t="inlineStr">
+        <is>
+          <t>{v}: escribe el mínimo y el máximo{e}.</t>
+        </is>
+      </c>
+      <c r="D678" s="6" t="inlineStr">
+        <is>
+          <t>{v}: enter the minimum and maximum{e}.</t>
+        </is>
+      </c>
+      <c r="E678" s="7" t="inlineStr"/>
+      <c r="F678" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes). Conservar {…} tal cual: se reemplaza por un dato</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B679" s="6" t="inlineStr">
+        <is>
+          <t>{v}: los valores deben estar entre {a} y {b}.</t>
+        </is>
+      </c>
+      <c r="C679" s="6" t="inlineStr">
+        <is>
+          <t>{v}: los valores deben estar entre {a} y {b}.</t>
+        </is>
+      </c>
+      <c r="D679" s="6" t="inlineStr">
+        <is>
+          <t>{v}: values must be between {a} and {b}.</t>
+        </is>
+      </c>
+      <c r="E679" s="7" t="inlineStr"/>
+      <c r="F679" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes). Conservar {…} tal cual: se reemplaza por un dato</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B680" s="6" t="inlineStr">
+        <is>
+          <t>{v}: el mínimo debe ser menor que el máximo{e}.</t>
+        </is>
+      </c>
+      <c r="C680" s="6" t="inlineStr">
+        <is>
+          <t>{v}: el mínimo debe ser menor que el máximo{e}.</t>
+        </is>
+      </c>
+      <c r="D680" s="6" t="inlineStr">
+        <is>
+          <t>{v}: the minimum must be lower than the maximum{e}.</t>
+        </is>
+      </c>
+      <c r="E680" s="7" t="inlineStr"/>
+      <c r="F680" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes). Conservar {…} tal cual: se reemplaza por un dato</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B681" s="6" t="inlineStr">
+        <is>
+          <t>(sistólica)</t>
+        </is>
+      </c>
+      <c r="C681" s="6" t="inlineStr">
+        <is>
+          <t>(sistólica)</t>
+        </is>
+      </c>
+      <c r="D681" s="6" t="inlineStr">
+        <is>
+          <t>(systolic)</t>
+        </is>
+      </c>
+      <c r="E681" s="7" t="inlineStr"/>
+      <c r="F681" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B682" s="6" t="inlineStr">
+        <is>
+          <t>(diastólica)</t>
+        </is>
+      </c>
+      <c r="C682" s="6" t="inlineStr">
+        <is>
+          <t>(diastólica)</t>
+        </is>
+      </c>
+      <c r="D682" s="6" t="inlineStr">
+        <is>
+          <t>(diastolic)</t>
+        </is>
+      </c>
+      <c r="E682" s="7" t="inlineStr"/>
+      <c r="F682" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B683" s="6" t="inlineStr">
+        <is>
+          <t>Plan de control guardado.</t>
+        </is>
+      </c>
+      <c r="C683" s="6" t="inlineStr">
+        <is>
+          <t>Plan de control guardado.</t>
+        </is>
+      </c>
+      <c r="D683" s="6" t="inlineStr">
+        <is>
+          <t>Monitoring plan saved.</t>
+        </is>
+      </c>
+      <c r="E683" s="7" t="inlineStr"/>
+      <c r="F683" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B684" s="6" t="inlineStr">
+        <is>
+          <t>Mínimo</t>
+        </is>
+      </c>
+      <c r="C684" s="6" t="inlineStr">
+        <is>
+          <t>Mínimo</t>
+        </is>
+      </c>
+      <c r="D684" s="6" t="inlineStr">
+        <is>
+          <t>Minimum</t>
+        </is>
+      </c>
+      <c r="E684" s="7" t="inlineStr"/>
+      <c r="F684" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B685" s="6" t="inlineStr">
+        <is>
+          <t>Máximo</t>
+        </is>
+      </c>
+      <c r="C685" s="6" t="inlineStr">
+        <is>
+          <t>Máximo</t>
+        </is>
+      </c>
+      <c r="D685" s="6" t="inlineStr">
+        <is>
+          <t>Maximum</t>
+        </is>
+      </c>
+      <c r="E685" s="7" t="inlineStr"/>
+      <c r="F685" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B686" s="6" t="inlineStr">
+        <is>
+          <t>Se le pide al paciente</t>
+        </is>
+      </c>
+      <c r="C686" s="6" t="inlineStr">
+        <is>
+          <t>Se le pide al paciente</t>
+        </is>
+      </c>
+      <c r="D686" s="6" t="inlineStr">
+        <is>
+          <t>Requested from the patient</t>
+        </is>
+      </c>
+      <c r="E686" s="7" t="inlineStr"/>
+      <c r="F686" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B687" s="6" t="inlineStr">
+        <is>
+          <t>No se le pide</t>
+        </is>
+      </c>
+      <c r="C687" s="6" t="inlineStr">
+        <is>
+          <t>No se le pide</t>
+        </is>
+      </c>
+      <c r="D687" s="6" t="inlineStr">
+        <is>
+          <t>Not requested</t>
+        </is>
+      </c>
+      <c r="E687" s="7" t="inlineStr"/>
+      <c r="F687" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B688" s="6" t="inlineStr">
+        <is>
+          <t>Sistólica (arriba)</t>
+        </is>
+      </c>
+      <c r="C688" s="6" t="inlineStr">
+        <is>
+          <t>Sistólica (arriba)</t>
+        </is>
+      </c>
+      <c r="D688" s="6" t="inlineStr">
+        <is>
+          <t>Systolic (top)</t>
+        </is>
+      </c>
+      <c r="E688" s="7" t="inlineStr"/>
+      <c r="F688" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B689" s="6" t="inlineStr">
+        <is>
+          <t>Rango normal</t>
+        </is>
+      </c>
+      <c r="C689" s="6" t="inlineStr">
+        <is>
+          <t>Rango normal</t>
+        </is>
+      </c>
+      <c r="D689" s="6" t="inlineStr">
+        <is>
+          <t>Normal range</t>
+        </is>
+      </c>
+      <c r="E689" s="7" t="inlineStr"/>
+      <c r="F689" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B690" s="6" t="inlineStr">
+        <is>
+          <t>Diastólica (abajo)</t>
+        </is>
+      </c>
+      <c r="C690" s="6" t="inlineStr">
+        <is>
+          <t>Diastólica (abajo)</t>
+        </is>
+      </c>
+      <c r="D690" s="6" t="inlineStr">
+        <is>
+          <t>Diastolic (bottom)</t>
+        </is>
+      </c>
+      <c r="E690" s="7" t="inlineStr"/>
+      <c r="F690" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B691" s="6" t="inlineStr">
+        <is>
+          <t>Meta (opcional)</t>
+        </is>
+      </c>
+      <c r="C691" s="6" t="inlineStr">
+        <is>
+          <t>Meta (opcional)</t>
+        </is>
+      </c>
+      <c r="D691" s="6" t="inlineStr">
+        <is>
+          <t>Goal (optional)</t>
+        </is>
+      </c>
+      <c r="E691" s="7" t="inlineStr"/>
+      <c r="F691" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B692" s="6" t="inlineStr">
+        <is>
+          <t>Ej. bajar a menos de 130/80 en 3 meses</t>
+        </is>
+      </c>
+      <c r="C692" s="6" t="inlineStr">
+        <is>
+          <t>Ej. bajar a menos de 130/80 en 3 meses</t>
+        </is>
+      </c>
+      <c r="D692" s="6" t="inlineStr">
+        <is>
+          <t>E.g. get below 130/80 in 3 months</t>
+        </is>
+      </c>
+      <c r="E692" s="7" t="inlineStr"/>
+      <c r="F692" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B693" s="6" t="inlineStr">
+        <is>
+          <t>Elige qué mediciones pedir, cada cuándo y en qué rango están bien. Fuera de rango, el registro avisa a tu equipo.</t>
+        </is>
+      </c>
+      <c r="C693" s="6" t="inlineStr">
+        <is>
+          <t>Elige qué mediciones pedir, cada cuándo y en qué rango están bien. Fuera de rango, el registro avisa a tu equipo.</t>
+        </is>
+      </c>
+      <c r="D693" s="6" t="inlineStr">
+        <is>
+          <t>Choose which measurements to request, how often and which range is fine. Out of range, the reading alerts your team.</t>
+        </is>
+      </c>
+      <c r="E693" s="7" t="inlineStr"/>
+      <c r="F693" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B694" s="6" t="inlineStr">
+        <is>
+          <t>Guardando…</t>
+        </is>
+      </c>
+      <c r="C694" s="6" t="inlineStr">
+        <is>
+          <t>Guardando…</t>
+        </is>
+      </c>
+      <c r="D694" s="6" t="inlineStr">
+        <is>
+          <t>Saving…</t>
+        </is>
+      </c>
+      <c r="E694" s="7" t="inlineStr"/>
+      <c r="F694" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B695" s="6" t="inlineStr">
+        <is>
+          <t>Guardar plan</t>
+        </is>
+      </c>
+      <c r="C695" s="6" t="inlineStr">
+        <is>
+          <t>Guardar plan</t>
+        </is>
+      </c>
+      <c r="D695" s="6" t="inlineStr">
+        <is>
+          <t>Save plan</t>
+        </is>
+      </c>
+      <c r="E695" s="7" t="inlineStr"/>
+      <c r="F695" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B696" s="6" t="inlineStr">
+        <is>
+          <t>No se recibió la versión del aviso de privacidad. Intenta más tarde.</t>
+        </is>
+      </c>
+      <c r="C696" s="6" t="inlineStr">
+        <is>
+          <t>No se recibió la versión del aviso de privacidad. Intenta más tarde.</t>
+        </is>
+      </c>
+      <c r="D696" s="6" t="inlineStr">
+        <is>
+          <t>The privacy notice version was not received. Try again later.</t>
+        </is>
+      </c>
+      <c r="E696" s="7" t="inlineStr"/>
+      <c r="F696" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B697" s="6" t="inlineStr">
+        <is>
+          <t>No se pudo cargar el aviso de privacidad. Sin él no se puede continuar.</t>
+        </is>
+      </c>
+      <c r="C697" s="6" t="inlineStr">
+        <is>
+          <t>No se pudo cargar el aviso de privacidad. Sin él no se puede continuar.</t>
+        </is>
+      </c>
+      <c r="D697" s="6" t="inlineStr">
+        <is>
+          <t>The privacy notice could not be loaded. You cannot continue without it.</t>
+        </is>
+      </c>
+      <c r="E697" s="7" t="inlineStr"/>
+      <c r="F697" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B698" s="6" t="inlineStr">
+        <is>
+          <t>Sin conexión. Mostramos lo último guardado ({fecha} {hora}).</t>
+        </is>
+      </c>
+      <c r="C698" s="6" t="inlineStr">
+        <is>
+          <t>Sin conexión. Mostramos lo último guardado ({fecha} {hora}).</t>
+        </is>
+      </c>
+      <c r="D698" s="6" t="inlineStr">
+        <is>
+          <t>No connection. Showing the last saved data ({fecha} {hora}).</t>
+        </is>
+      </c>
+      <c r="E698" s="7" t="inlineStr"/>
+      <c r="F698" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes). Conservar {…} tal cual: se reemplaza por un dato</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B699" s="6" t="inlineStr">
+        <is>
+          <t>Hoy no tienes tomas de medicamento.</t>
+        </is>
+      </c>
+      <c r="C699" s="6" t="inlineStr">
+        <is>
+          <t>Hoy no tienes tomas de medicamento.</t>
+        </is>
+      </c>
+      <c r="D699" s="6" t="inlineStr">
+        <is>
+          <t>You have no medication doses today.</t>
+        </is>
+      </c>
+      <c r="E699" s="7" t="inlineStr"/>
+      <c r="F699" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B700" s="6" t="inlineStr">
+        <is>
+          <t>¿Tu presión de arriba es {n}?</t>
+        </is>
+      </c>
+      <c r="C700" s="6" t="inlineStr">
+        <is>
+          <t>¿Tu presión de arriba es {n}?</t>
+        </is>
+      </c>
+      <c r="D700" s="6" t="inlineStr">
+        <is>
+          <t>Is your top blood pressure number {n}?</t>
+        </is>
+      </c>
+      <c r="E700" s="7" t="inlineStr"/>
+      <c r="F700" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes). Conservar {…} tal cual: se reemplaza por un dato</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B701" s="6" t="inlineStr">
+        <is>
+          <t>¿Tu presión de abajo es {n}?</t>
+        </is>
+      </c>
+      <c r="C701" s="6" t="inlineStr">
+        <is>
+          <t>¿Tu presión de abajo es {n}?</t>
+        </is>
+      </c>
+      <c r="D701" s="6" t="inlineStr">
+        <is>
+          <t>Is your bottom blood pressure number {n}?</t>
+        </is>
+      </c>
+      <c r="E701" s="7" t="inlineStr"/>
+      <c r="F701" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes). Conservar {…} tal cual: se reemplaza por un dato</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B702" s="6" t="inlineStr">
+        <is>
+          <t>¿Tu {v} es {n} {u}?</t>
+        </is>
+      </c>
+      <c r="C702" s="6" t="inlineStr">
+        <is>
+          <t>¿Tu {v} es {n} {u}?</t>
+        </is>
+      </c>
+      <c r="D702" s="6" t="inlineStr">
+        <is>
+          <t>Is your {v} {n} {u}?</t>
+        </is>
+      </c>
+      <c r="E702" s="7" t="inlineStr"/>
+      <c r="F702" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes). Conservar {…} tal cual: se reemplaza por un dato</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B703" s="6" t="inlineStr">
+        <is>
+          <t>Revisa el número</t>
+        </is>
+      </c>
+      <c r="C703" s="6" t="inlineStr">
+        <is>
+          <t>Revisa el número</t>
+        </is>
+      </c>
+      <c r="D703" s="6" t="inlineStr">
+        <is>
+          <t>Check the number</t>
+        </is>
+      </c>
+      <c r="E703" s="7" t="inlineStr"/>
+      <c r="F703" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B704" s="6" t="inlineStr">
+        <is>
+          <t>Si es correcto, confírmalo; si no, corrígelo.</t>
+        </is>
+      </c>
+      <c r="C704" s="6" t="inlineStr">
+        <is>
+          <t>Si es correcto, confírmalo; si no, corrígelo.</t>
+        </is>
+      </c>
+      <c r="D704" s="6" t="inlineStr">
+        <is>
+          <t>If it is correct, confirm it; if not, fix it.</t>
+        </is>
+      </c>
+      <c r="E704" s="7" t="inlineStr"/>
+      <c r="F704" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B705" s="6" t="inlineStr">
+        <is>
+          <t>Sí, es correcto</t>
+        </is>
+      </c>
+      <c r="C705" s="6" t="inlineStr">
+        <is>
+          <t>Sí, es correcto</t>
+        </is>
+      </c>
+      <c r="D705" s="6" t="inlineStr">
+        <is>
+          <t>Yes, it is correct</t>
+        </is>
+      </c>
+      <c r="E705" s="7" t="inlineStr"/>
+      <c r="F705" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B706" s="6" t="inlineStr">
+        <is>
+          <t>Corregir</t>
+        </is>
+      </c>
+      <c r="C706" s="6" t="inlineStr">
+        <is>
+          <t>Corregir</t>
+        </is>
+      </c>
+      <c r="D706" s="6" t="inlineStr">
+        <is>
+          <t>Fix it</t>
+        </is>
+      </c>
+      <c r="E706" s="7" t="inlineStr"/>
+      <c r="F706" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B707" s="6" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="C707" s="6" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="D707" s="6" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="E707" s="7" t="inlineStr"/>
+      <c r="F707" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B708" s="6" t="inlineStr">
+        <is>
+          <t>¿Salir de la receta?</t>
+        </is>
+      </c>
+      <c r="C708" s="6" t="inlineStr">
+        <is>
+          <t>¿Salir de la receta?</t>
+        </is>
+      </c>
+      <c r="D708" s="6" t="inlineStr">
+        <is>
+          <t>Leave the prescription?</t>
+        </is>
+      </c>
+      <c r="E708" s="7" t="inlineStr"/>
+      <c r="F708" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B709" s="6" t="inlineStr">
+        <is>
+          <t>Se perderá lo que ya se leyó y revisaste.</t>
+        </is>
+      </c>
+      <c r="C709" s="6" t="inlineStr">
+        <is>
+          <t>Se perderá lo que ya se leyó y revisaste.</t>
+        </is>
+      </c>
+      <c r="D709" s="6" t="inlineStr">
+        <is>
+          <t>What was read and what you reviewed will be lost.</t>
+        </is>
+      </c>
+      <c r="E709" s="7" t="inlineStr"/>
+      <c r="F709" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B710" s="6" t="inlineStr">
+        <is>
+          <t>Salir</t>
+        </is>
+      </c>
+      <c r="C710" s="6" t="inlineStr">
+        <is>
+          <t>Salir</t>
+        </is>
+      </c>
+      <c r="D710" s="6" t="inlineStr">
+        <is>
+          <t>Leave</t>
+        </is>
+      </c>
+      <c r="E710" s="7" t="inlineStr"/>
+      <c r="F710" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B711" s="6" t="inlineStr">
+        <is>
+          <t>Seguir aquí</t>
+        </is>
+      </c>
+      <c r="C711" s="6" t="inlineStr">
+        <is>
+          <t>Seguir aquí</t>
+        </is>
+      </c>
+      <c r="D711" s="6" t="inlineStr">
+        <is>
+          <t>Stay here</t>
+        </is>
+      </c>
+      <c r="E711" s="7" t="inlineStr"/>
+      <c r="F711" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B712" s="6" t="inlineStr">
+        <is>
+          <t>SENDA está bloqueada</t>
+        </is>
+      </c>
+      <c r="C712" s="6" t="inlineStr">
+        <is>
+          <t>SENDA está bloqueada</t>
+        </is>
+      </c>
+      <c r="D712" s="6" t="inlineStr">
+        <is>
+          <t>SENDA is locked</t>
+        </is>
+      </c>
+      <c r="E712" s="7" t="inlineStr"/>
+      <c r="F712" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B713" s="6" t="inlineStr">
+        <is>
+          <t>Desbloquear</t>
+        </is>
+      </c>
+      <c r="C713" s="6" t="inlineStr">
+        <is>
+          <t>Desbloquear</t>
+        </is>
+      </c>
+      <c r="D713" s="6" t="inlineStr">
+        <is>
+          <t>Unlock</t>
+        </is>
+      </c>
+      <c r="E713" s="7" t="inlineStr"/>
+      <c r="F713" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B714" s="6" t="inlineStr">
+        <is>
+          <t>Entrar con contraseña</t>
+        </is>
+      </c>
+      <c r="C714" s="6" t="inlineStr">
+        <is>
+          <t>Entrar con contraseña</t>
+        </is>
+      </c>
+      <c r="D714" s="6" t="inlineStr">
+        <is>
+          <t>Log in with password</t>
+        </is>
+      </c>
+      <c r="E714" s="7" t="inlineStr"/>
+      <c r="F714" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B715" s="6" t="inlineStr">
+        <is>
+          <t>No se pudo reproducir el audio. Revisa tu internet.</t>
+        </is>
+      </c>
+      <c r="C715" s="6" t="inlineStr">
+        <is>
+          <t>No se pudo reproducir el audio. Revisa tu internet.</t>
+        </is>
+      </c>
+      <c r="D715" s="6" t="inlineStr">
+        <is>
+          <t>Could not play the audio. Check your internet.</t>
+        </is>
+      </c>
+      <c r="E715" s="7" t="inlineStr"/>
+      <c r="F715" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B716" s="6" t="inlineStr">
+        <is>
+          <t>Instala la voz en inglés en los Ajustes del teléfono para escuchar.</t>
+        </is>
+      </c>
+      <c r="C716" s="6" t="inlineStr">
+        <is>
+          <t>Instala la voz en inglés en los Ajustes del teléfono para escuchar.</t>
+        </is>
+      </c>
+      <c r="D716" s="6" t="inlineStr">
+        <is>
+          <t>Install the English voice in your phone Settings to listen.</t>
+        </is>
+      </c>
+      <c r="E716" s="7" t="inlineStr"/>
+      <c r="F716" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B717" s="6" t="inlineStr">
+        <is>
+          <t>Instala la voz en español en los Ajustes del teléfono para escuchar.</t>
+        </is>
+      </c>
+      <c r="C717" s="6" t="inlineStr">
+        <is>
+          <t>Instala la voz en español en los Ajustes del teléfono para escuchar.</t>
+        </is>
+      </c>
+      <c r="D717" s="6" t="inlineStr">
+        <is>
+          <t>Install the Spanish voice in your phone Settings to listen.</t>
+        </is>
+      </c>
+      <c r="E717" s="7" t="inlineStr"/>
+      <c r="F717" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="6" t="inlineStr">
+        <is>
+          <t>Texto de pantalla</t>
+        </is>
+      </c>
+      <c r="B718" s="6" t="inlineStr">
+        <is>
+          <t>No se pudo leer en voz alta.</t>
+        </is>
+      </c>
+      <c r="C718" s="6" t="inlineStr">
+        <is>
+          <t>No se pudo leer en voz alta.</t>
+        </is>
+      </c>
+      <c r="D718" s="6" t="inlineStr">
+        <is>
+          <t>Could not read aloud.</t>
+        </is>
+      </c>
+      <c r="E718" s="7" t="inlineStr"/>
+      <c r="F718" s="6" t="inlineStr">
+        <is>
+          <t>Nuevo (Android/iOS y pendientes)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F615"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>